<commit_message>
summary ui,result ui,download pdf
</commit_message>
<xml_diff>
--- a/public/templates/fuel-template.xlsx
+++ b/public/templates/fuel-template.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Hackathon\ESGroww\ESGroww\public\templates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Karthika\Desktop\ESGroww\ESGroww\public\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CEF1354F-8AD9-451D-98BD-D8A803A795BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A56AF156-EFC8-4DE0-B617-8B45FFF20930}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{4FF0677B-3B9D-4E7D-A727-B3763C791967}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{4FF0677B-3B9D-4E7D-A727-B3763C791967}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,15 +39,6 @@
     <t>dgDieselLitres</t>
   </si>
   <si>
-    <t>⛽  Fuel / DG Consumption Upload Template</t>
-  </si>
-  <si>
-    <t>month</t>
-  </si>
-  <si>
-    <t>year</t>
-  </si>
-  <si>
     <t>DG_Runtime_Hours</t>
   </si>
   <si>
@@ -73,6 +64,15 @@
   </si>
   <si>
     <t>Quantity of piped natural gas (PNG) or compressed natural gas (CNG) consumed, in kg. Enter 0 if not applicable.</t>
+  </si>
+  <si>
+    <t>Month</t>
+  </si>
+  <si>
+    <t>Year</t>
+  </si>
+  <si>
+    <t>⛽  Fuel Consumption Upload Template</t>
   </si>
 </sst>
 </file>
@@ -161,14 +161,14 @@
   </cellStyleXfs>
   <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -495,53 +495,53 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="18" x14ac:dyDescent="0.35">
-      <c r="A1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
+      <c r="A1" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B1" s="3"/>
+      <c r="C1" s="3"/>
+      <c r="D1" s="3"/>
+      <c r="E1" s="3"/>
+      <c r="F1" s="3"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="E2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="F2" s="1" t="s">
         <v>3</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>6</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="72" x14ac:dyDescent="0.35">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D3" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="E3" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="F3" s="2" t="s">
         <v>9</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>